<commit_message>
Auto: Analysis complete | Temp: Ambient | Max Cycle: 148 | Anomalies: 0 | 2026-04-23 10:37
</commit_message>
<xml_diff>
--- a/reports/Master_Retention_Summary.xlsx
+++ b/reports/Master_Retention_Summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F403"/>
+  <dimension ref="A1:F446"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10108,6 +10108,1038 @@
         <v>96.25435531652923</v>
       </c>
     </row>
+    <row r="404">
+      <c r="A404" t="n">
+        <v>54</v>
+      </c>
+      <c r="B404" t="n">
+        <v>1.061577545637317</v>
+      </c>
+      <c r="C404" t="n">
+        <v>1.061577545637317</v>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F404" t="n">
+        <v>96.50704960339246</v>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="n">
+        <v>55</v>
+      </c>
+      <c r="B405" t="n">
+        <v>2.164289885491261</v>
+      </c>
+      <c r="C405" t="n">
+        <v>1.102712339853944</v>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F405" t="n">
+        <v>100.2465763503585</v>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="n">
+        <v>56</v>
+      </c>
+      <c r="B406" t="n">
+        <v>3.267583323939062</v>
+      </c>
+      <c r="C406" t="n">
+        <v>1.103293438447801</v>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E406" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F406" t="n">
+        <v>100.2994034952546</v>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="n">
+        <v>57</v>
+      </c>
+      <c r="B407" t="n">
+        <v>4.372056985656962</v>
+      </c>
+      <c r="C407" t="n">
+        <v>1.1044736617179</v>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F407" t="n">
+        <v>100.4066965198091</v>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="n">
+        <v>58</v>
+      </c>
+      <c r="B408" t="n">
+        <v>5.473847553432576</v>
+      </c>
+      <c r="C408" t="n">
+        <v>1.101790567775614</v>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F408" t="n">
+        <v>100.1627788886922</v>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="n">
+        <v>59</v>
+      </c>
+      <c r="B409" t="n">
+        <v>6.565619223003772</v>
+      </c>
+      <c r="C409" t="n">
+        <v>1.091771669571195</v>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F409" t="n">
+        <v>99.25196996101776</v>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="n">
+        <v>60</v>
+      </c>
+      <c r="B410" t="n">
+        <v>7.653588180894634</v>
+      </c>
+      <c r="C410" t="n">
+        <v>1.087968957890863</v>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E410" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F410" t="n">
+        <v>98.90626889916932</v>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="n">
+        <v>61</v>
+      </c>
+      <c r="B411" t="n">
+        <v>8.739329367509095</v>
+      </c>
+      <c r="C411" t="n">
+        <v>1.08574118661446</v>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F411" t="n">
+        <v>98.70374423767821</v>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="n">
+        <v>62</v>
+      </c>
+      <c r="B412" t="n">
+        <v>9.819657743935954</v>
+      </c>
+      <c r="C412" t="n">
+        <v>1.080328376426859</v>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F412" t="n">
+        <v>98.21167058425992</v>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="n">
+        <v>63</v>
+      </c>
+      <c r="B413" t="n">
+        <v>10.90013606510165</v>
+      </c>
+      <c r="C413" t="n">
+        <v>1.080478321165694</v>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E413" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F413" t="n">
+        <v>98.22530192415402</v>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="n">
+        <v>64</v>
+      </c>
+      <c r="B414" t="n">
+        <v>11.9795786581839</v>
+      </c>
+      <c r="C414" t="n">
+        <v>1.079442593082256</v>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F414" t="n">
+        <v>98.13114482565959</v>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="n">
+        <v>65</v>
+      </c>
+      <c r="B415" t="n">
+        <v>13.05247552649116</v>
+      </c>
+      <c r="C415" t="n">
+        <v>1.072896868307252</v>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E415" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F415" t="n">
+        <v>97.53607893702289</v>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="n">
+        <v>66</v>
+      </c>
+      <c r="B416" t="n">
+        <v>14.12108721883883</v>
+      </c>
+      <c r="C416" t="n">
+        <v>1.068611692347671</v>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F416" t="n">
+        <v>97.14651748615194</v>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="n">
+        <v>67</v>
+      </c>
+      <c r="B417" t="n">
+        <v>15.18801044751135</v>
+      </c>
+      <c r="C417" t="n">
+        <v>1.066923228672525</v>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E417" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F417" t="n">
+        <v>96.9930207884114</v>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="n">
+        <v>68</v>
+      </c>
+      <c r="B418" t="n">
+        <v>16.25279605790751</v>
+      </c>
+      <c r="C418" t="n">
+        <v>1.064785610396154</v>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E418" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F418" t="n">
+        <v>96.79869185419578</v>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="n">
+        <v>69</v>
+      </c>
+      <c r="B419" t="n">
+        <v>17.14256780443614</v>
+      </c>
+      <c r="C419" t="n">
+        <v>0.8897717465286341</v>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F419" t="n">
+        <v>80.88834059351218</v>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="n">
+        <v>70</v>
+      </c>
+      <c r="B420" t="n">
+        <v>18.20948826116475</v>
+      </c>
+      <c r="C420" t="n">
+        <v>1.066920456728607</v>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E420" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F420" t="n">
+        <v>96.99276879350968</v>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="n">
+        <v>71</v>
+      </c>
+      <c r="B421" t="n">
+        <v>19.2714905333444</v>
+      </c>
+      <c r="C421" t="n">
+        <v>1.062002272179654</v>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E421" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F421" t="n">
+        <v>96.54566110724132</v>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="n">
+        <v>72</v>
+      </c>
+      <c r="B422" t="n">
+        <v>20.33037048751444</v>
+      </c>
+      <c r="C422" t="n">
+        <v>1.058879954170042</v>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E422" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F422" t="n">
+        <v>96.26181401545834</v>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="n">
+        <v>73</v>
+      </c>
+      <c r="B423" t="n">
+        <v>21.38314339519933</v>
+      </c>
+      <c r="C423" t="n">
+        <v>1.052772907684886</v>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E423" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F423" t="n">
+        <v>95.7066279713533</v>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="n">
+        <v>74</v>
+      </c>
+      <c r="B424" t="n">
+        <v>22.43621759374313</v>
+      </c>
+      <c r="C424" t="n">
+        <v>1.053074198543797</v>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E424" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F424" t="n">
+        <v>95.73401804943609</v>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="n">
+        <v>75</v>
+      </c>
+      <c r="B425" t="n">
+        <v>23.48822786663382</v>
+      </c>
+      <c r="C425" t="n">
+        <v>1.052010272890691</v>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F425" t="n">
+        <v>95.63729753551732</v>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="n">
+        <v>76</v>
+      </c>
+      <c r="B426" t="n">
+        <v>24.53769265857875</v>
+      </c>
+      <c r="C426" t="n">
+        <v>1.049464791944928</v>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F426" t="n">
+        <v>95.40589017681161</v>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="n">
+        <v>77</v>
+      </c>
+      <c r="B427" t="n">
+        <v>25.59265457381279</v>
+      </c>
+      <c r="C427" t="n">
+        <v>1.054961915234045</v>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F427" t="n">
+        <v>95.90562865764049</v>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="n">
+        <v>78</v>
+      </c>
+      <c r="B428" t="n">
+        <v>26.64747142294459</v>
+      </c>
+      <c r="C428" t="n">
+        <v>1.0548168491318</v>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F428" t="n">
+        <v>95.89244083016365</v>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="n">
+        <v>79</v>
+      </c>
+      <c r="B429" t="n">
+        <v>27.70105142219042</v>
+      </c>
+      <c r="C429" t="n">
+        <v>1.053579999245834</v>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F429" t="n">
+        <v>95.77999993143942</v>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="n">
+        <v>80</v>
+      </c>
+      <c r="B430" t="n">
+        <v>28.75368506607596</v>
+      </c>
+      <c r="C430" t="n">
+        <v>1.052633643885539</v>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E430" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F430" t="n">
+        <v>95.69396762595807</v>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="n">
+        <v>81</v>
+      </c>
+      <c r="B431" t="n">
+        <v>29.80563104953838</v>
+      </c>
+      <c r="C431" t="n">
+        <v>1.051945983462417</v>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F431" t="n">
+        <v>95.63145304203792</v>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="n">
+        <v>82</v>
+      </c>
+      <c r="B432" t="n">
+        <v>30.8575977483636</v>
+      </c>
+      <c r="C432" t="n">
+        <v>1.051966698825215</v>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E432" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F432" t="n">
+        <v>95.63333625683769</v>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="n">
+        <v>83</v>
+      </c>
+      <c r="B433" t="n">
+        <v>31.90853479851857</v>
+      </c>
+      <c r="C433" t="n">
+        <v>1.050937050154975</v>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F433" t="n">
+        <v>95.53973183227042</v>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="n">
+        <v>84</v>
+      </c>
+      <c r="B434" t="n">
+        <v>32.95801188122525</v>
+      </c>
+      <c r="C434" t="n">
+        <v>1.049477082706677</v>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E434" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F434" t="n">
+        <v>95.40700751878877</v>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="n">
+        <v>85</v>
+      </c>
+      <c r="B435" t="n">
+        <v>34.00615073531269</v>
+      </c>
+      <c r="C435" t="n">
+        <v>1.048138854087448</v>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F435" t="n">
+        <v>95.28535037158615</v>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="n">
+        <v>86</v>
+      </c>
+      <c r="B436" t="n">
+        <v>35.05383725842688</v>
+      </c>
+      <c r="C436" t="n">
+        <v>1.047686523114187</v>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E436" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F436" t="n">
+        <v>95.24422937401701</v>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="n">
+        <v>87</v>
+      </c>
+      <c r="B437" t="n">
+        <v>36.10048850578645</v>
+      </c>
+      <c r="C437" t="n">
+        <v>1.04665124735957</v>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E437" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F437" t="n">
+        <v>95.15011339632453</v>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="n">
+        <v>88</v>
+      </c>
+      <c r="B438" t="n">
+        <v>36.98470135955655</v>
+      </c>
+      <c r="C438" t="n">
+        <v>0.8842128537701015</v>
+      </c>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E438" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F438" t="n">
+        <v>80.38298670637286</v>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="n">
+        <v>89</v>
+      </c>
+      <c r="B439" t="n">
+        <v>38.03563074689517</v>
+      </c>
+      <c r="C439" t="n">
+        <v>1.050929387338613</v>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F439" t="n">
+        <v>95.53903521260115</v>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="n">
+        <v>90</v>
+      </c>
+      <c r="B440" t="n">
+        <v>39.08096058531849</v>
+      </c>
+      <c r="C440" t="n">
+        <v>1.045329838423321</v>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E440" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F440" t="n">
+        <v>95.02998531121096</v>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="n">
+        <v>91</v>
+      </c>
+      <c r="B441" t="n">
+        <v>40.124614391113</v>
+      </c>
+      <c r="C441" t="n">
+        <v>1.043653805794513</v>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F441" t="n">
+        <v>94.87761870859207</v>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="n">
+        <v>92</v>
+      </c>
+      <c r="B442" t="n">
+        <v>41.16745894009971</v>
+      </c>
+      <c r="C442" t="n">
+        <v>1.042844548986714</v>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E442" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F442" t="n">
+        <v>94.80404990788313</v>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="n">
+        <v>93</v>
+      </c>
+      <c r="B443" t="n">
+        <v>42.20830582705204</v>
+      </c>
+      <c r="C443" t="n">
+        <v>1.040846886952323</v>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F443" t="n">
+        <v>94.62244426839302</v>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="n">
+        <v>94</v>
+      </c>
+      <c r="B444" t="n">
+        <v>43.23699830529267</v>
+      </c>
+      <c r="C444" t="n">
+        <v>1.028692478240629</v>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E444" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F444" t="n">
+        <v>93.51749802187534</v>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="n">
+        <v>95</v>
+      </c>
+      <c r="B445" t="n">
+        <v>44.26474272593617</v>
+      </c>
+      <c r="C445" t="n">
+        <v>1.027744420643508</v>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F445" t="n">
+        <v>93.43131096759161</v>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="n">
+        <v>96</v>
+      </c>
+      <c r="B446" t="n">
+        <v>45.29112759404217</v>
+      </c>
+      <c r="C446" t="n">
+        <v>1.026384868105993</v>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E446" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F446" t="n">
+        <v>93.30771528236296</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: Analysis complete | Temp: Ambient | Max Cycle: 2 | Anomalies: 0 | 2026-04-23 10:58
</commit_message>
<xml_diff>
--- a/reports/Master_Retention_Summary.xlsx
+++ b/reports/Master_Retention_Summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -486,17 +486,17 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>1.160620725192767</v>
+        <v>1.138645812632654</v>
       </c>
       <c r="C3" t="n">
-        <v>1.160620725192767</v>
+        <v>1.138645812632654</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>CS2_36</t>
+          <t>CS2_35</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -505,7 +505,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>105.5109750175243</v>
+        <v>103.5132556938776</v>
       </c>
     </row>
     <row r="4">
@@ -513,14 +513,14 @@
         <v>1</v>
       </c>
       <c r="B4" t="n">
-        <v>1.153332504667897</v>
+        <v>1.160620725192767</v>
       </c>
       <c r="C4" t="n">
-        <v>1.153332504667897</v>
+        <v>1.160620725192767</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>CS2_37</t>
+          <t>CS2_36</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>104.8484095152634</v>
+        <v>105.5109750175243</v>
       </c>
     </row>
     <row r="5">
@@ -537,22 +537,46 @@
         <v>1</v>
       </c>
       <c r="B5" t="n">
+        <v>1.153332504667897</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1.153332504667897</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>CS2_37</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>104.8484095152634</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" t="n">
         <v>1.16241194625815</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C6" t="n">
         <v>1.16241194625815</v>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>CS2_38</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>Ambient</t>
         </is>
       </c>
-      <c r="F5" t="n">
+      <c r="F6" t="n">
         <v>105.6738132961954</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto: Analysis complete | Temp: Ambient | Max Cycle: 2 | Anomalies: 0 | 2026-04-23 10:59
</commit_message>
<xml_diff>
--- a/reports/Master_Retention_Summary.xlsx
+++ b/reports/Master_Retention_Summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -628,6 +628,30 @@
         <v>105.6738132961954</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" t="n">
+        <v>1.140773820517232</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1.140773820517232</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>103.706710956112</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: Analysis complete | Temp: Ambient | Max Cycle: 3 | Anomalies: 0 | 2026-04-23 15:32
</commit_message>
<xml_diff>
--- a/reports/Master_Retention_Summary.xlsx
+++ b/reports/Master_Retention_Summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -652,6 +652,30 @@
         <v>103.706710956112</v>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>3</v>
+      </c>
+      <c r="B10" t="n">
+        <v>1.139105930615482</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1.139105930615482</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>103.5550846014075</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: Analysis complete | Temp: Ambient | Max Cycle: 47 | Anomalies: 0 | 2026-04-24 12:02
</commit_message>
<xml_diff>
--- a/reports/Master_Retention_Summary.xlsx
+++ b/reports/Master_Retention_Summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -510,17 +510,17 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>1.160620725192767</v>
+        <v>1.052322023911945</v>
       </c>
       <c r="C4" t="n">
-        <v>1.160620725192767</v>
+        <v>1.052322023911945</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>CS2_36</t>
+          <t>CS2_35</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -529,22 +529,22 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>105.5109750175243</v>
+        <v>95.66563853744955</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>1.145706012058183</v>
+        <v>2.149665492833128</v>
       </c>
       <c r="C5" t="n">
-        <v>1.145706012058183</v>
+        <v>1.097343468921183</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>CS2_36</t>
+          <t>CS2_35</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -553,22 +553,22 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>104.1550920052894</v>
+        <v>99.75849717465297</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>1.153332504667897</v>
+        <v>3.245035743823332</v>
       </c>
       <c r="C6" t="n">
-        <v>1.153332504667897</v>
+        <v>1.095370250990204</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>CS2_37</t>
+          <t>CS2_35</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -577,22 +577,22 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>104.8484095152634</v>
+        <v>99.57911372638219</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>1.134444845802931</v>
+        <v>4.3427396829912</v>
       </c>
       <c r="C7" t="n">
-        <v>1.134444845802931</v>
+        <v>1.097703939167868</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>CS2_37</t>
+          <t>CS2_35</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -601,22 +601,22 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>103.1313496184483</v>
+        <v>99.79126719707895</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>1.16241194625815</v>
+        <v>5.438155466960088</v>
       </c>
       <c r="C8" t="n">
-        <v>1.16241194625815</v>
+        <v>1.095415783968887</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>CS2_38</t>
+          <t>CS2_35</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -625,22 +625,22 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>105.6738132961954</v>
+        <v>99.58325308808065</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>1.140773820517232</v>
+        <v>6.408604373024617</v>
       </c>
       <c r="C9" t="n">
-        <v>1.140773820517232</v>
+        <v>0.9704489060645294</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>CS2_38</t>
+          <t>CS2_35</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -649,30 +649,1110 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>103.706710956112</v>
+        <v>88.22262782404812</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="n">
+        <v>7.495652225355175</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1.087047852330558</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>98.82253203005074</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="n">
+        <v>8.577396784697651</v>
+      </c>
+      <c r="C11" t="n">
+        <v>1.081744559342476</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>98.34041448567962</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="n">
+        <v>9.654946259914045</v>
+      </c>
+      <c r="C12" t="n">
+        <v>1.077549475216394</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>97.95904320149033</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="n">
+        <v>10.72613836450355</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1.071192104589505</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>97.38110041722771</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="n">
+        <v>11.79860684954863</v>
+      </c>
+      <c r="C14" t="n">
+        <v>1.072468485045077</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>97.49713500409788</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="n">
+        <v>12.86786434001764</v>
+      </c>
+      <c r="C15" t="n">
+        <v>1.069257490469012</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>97.20522640627377</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="n">
+        <v>13.9297296638013</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1.061865323783662</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>96.53321125306019</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="n">
+        <v>14.98952004353151</v>
+      </c>
+      <c r="C17" t="n">
+        <v>1.05979037973021</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>96.34457997547359</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="n">
+        <v>16.04749855873573</v>
+      </c>
+      <c r="C18" t="n">
+        <v>1.057978515204223</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>96.17986501856569</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="n">
+        <v>17.10340536937683</v>
+      </c>
+      <c r="C19" t="n">
+        <v>1.055906810641098</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>95.99152824009978</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="n">
+        <v>18.1556290521891</v>
+      </c>
+      <c r="C20" t="n">
+        <v>1.052223682812269</v>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>95.65669843747897</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="n">
+        <v>19.20997154058639</v>
+      </c>
+      <c r="C21" t="n">
+        <v>1.054342488397296</v>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>95.84931712702691</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="n">
+        <v>20.26299732771692</v>
+      </c>
+      <c r="C22" t="n">
+        <v>1.053025787130522</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>95.72961701186567</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="n">
+        <v>21.31033341195971</v>
+      </c>
+      <c r="C23" t="n">
+        <v>1.047336084242794</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>95.21237129479941</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="n">
+        <v>22.35610598333428</v>
+      </c>
+      <c r="C24" t="n">
+        <v>1.045772571374567</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>95.07023376132425</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="n">
+        <v>23.40056677922347</v>
+      </c>
+      <c r="C25" t="n">
+        <v>1.044460795889197</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>94.95098144447246</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="n">
+        <v>24.44359582009594</v>
+      </c>
+      <c r="C26" t="n">
+        <v>1.043029040872465</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>94.82082189749683</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="n">
+        <v>25.4831948218273</v>
+      </c>
+      <c r="C27" t="n">
+        <v>1.039599001731357</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>94.5090001573961</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="n">
+        <v>26.52631445530069</v>
+      </c>
+      <c r="C28" t="n">
+        <v>1.043119633473388</v>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>94.82905758848985</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="n">
+        <v>27.5686670992941</v>
+      </c>
+      <c r="C29" t="n">
+        <v>1.042352643993418</v>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>94.75933127212889</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="n">
+        <v>28.60979222529076</v>
+      </c>
+      <c r="C30" t="n">
+        <v>1.041125125996658</v>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>94.64773872696887</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="n">
+        <v>29.64938541586051</v>
+      </c>
+      <c r="C31" t="n">
+        <v>1.03959319056975</v>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>94.50847186997728</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="n">
+        <v>30.68792447367722</v>
+      </c>
+      <c r="C32" t="n">
+        <v>1.038539057816706</v>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>94.41264161970055</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="n">
+        <v>31.7263162152612</v>
+      </c>
+      <c r="C33" t="n">
+        <v>1.038391741583983</v>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>94.39924923490749</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="n">
+        <v>32.76338812831584</v>
+      </c>
+      <c r="C34" t="n">
+        <v>1.037071913054639</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>94.27926482314901</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="n">
+        <v>33.7987298481729</v>
+      </c>
+      <c r="C35" t="n">
+        <v>1.035341719857065</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>94.12197453246048</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="n">
+        <v>34.83270037940027</v>
+      </c>
+      <c r="C36" t="n">
+        <v>1.033970531227368</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>93.9973210206698</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="n">
+        <v>35.86574666724295</v>
+      </c>
+      <c r="C37" t="n">
+        <v>1.033046287842673</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>93.91329889478844</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="n">
+        <v>36.89740618197521</v>
+      </c>
+      <c r="C38" t="n">
+        <v>1.031659514732269</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>93.78722861202442</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="n">
+        <v>37.92829661484846</v>
+      </c>
+      <c r="C39" t="n">
+        <v>1.030890432873242</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>93.71731207938568</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="n">
+        <v>38.95850830029624</v>
+      </c>
+      <c r="C40" t="n">
+        <v>1.030211685447789</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>93.65560776798078</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="n">
+        <v>39.98860228884588</v>
+      </c>
+      <c r="C41" t="n">
+        <v>1.030093988549631</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>93.6449080499664</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="n">
+        <v>41.01705848167371</v>
+      </c>
+      <c r="C42" t="n">
+        <v>1.028456192827839</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>93.49601752980357</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="n">
+        <v>42.04438475344786</v>
+      </c>
+      <c r="C43" t="n">
+        <v>1.027326271774143</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>93.39329743401301</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="n">
+        <v>43.07010828743945</v>
+      </c>
+      <c r="C44" t="n">
+        <v>1.025723533991588</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>93.24759399923526</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="n">
+        <v>44.08658300417674</v>
+      </c>
+      <c r="C45" t="n">
+        <v>1.016474716737292</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>92.40679243066293</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="n">
+        <v>45.10024541836556</v>
+      </c>
+      <c r="C46" t="n">
+        <v>1.013662414188822</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>92.15112856262017</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="n">
+        <v>46.1126554106551</v>
+      </c>
+      <c r="C47" t="n">
+        <v>1.012409992289541</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>92.03727202632192</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="n">
+        <v>46.39238602108801</v>
+      </c>
+      <c r="C48" t="n">
+        <v>0.2797306104329067</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>25.4300554939006</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>1</v>
+      </c>
+      <c r="B49" t="n">
+        <v>1.160620725192767</v>
+      </c>
+      <c r="C49" t="n">
+        <v>1.160620725192767</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>CS2_36</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>105.5109750175243</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>2</v>
+      </c>
+      <c r="B50" t="n">
+        <v>1.145706012058183</v>
+      </c>
+      <c r="C50" t="n">
+        <v>1.145706012058183</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>CS2_36</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>104.1550920052894</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>1</v>
+      </c>
+      <c r="B51" t="n">
+        <v>1.153332504667897</v>
+      </c>
+      <c r="C51" t="n">
+        <v>1.153332504667897</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>CS2_37</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>104.8484095152634</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>2</v>
+      </c>
+      <c r="B52" t="n">
+        <v>1.134444845802931</v>
+      </c>
+      <c r="C52" t="n">
+        <v>1.134444845802931</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>CS2_37</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>103.1313496184483</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>1</v>
+      </c>
+      <c r="B53" t="n">
+        <v>1.16241194625815</v>
+      </c>
+      <c r="C53" t="n">
+        <v>1.16241194625815</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F53" t="n">
+        <v>105.6738132961954</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>2</v>
+      </c>
+      <c r="B54" t="n">
+        <v>1.140773820517232</v>
+      </c>
+      <c r="C54" t="n">
+        <v>1.140773820517232</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F54" t="n">
+        <v>103.706710956112</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
         <v>3</v>
       </c>
-      <c r="B10" t="n">
+      <c r="B55" t="n">
         <v>1.139105930615482</v>
       </c>
-      <c r="C10" t="n">
+      <c r="C55" t="n">
         <v>1.139105930615482</v>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D55" t="inlineStr">
         <is>
           <t>CS2_38</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>Ambient</t>
-        </is>
-      </c>
-      <c r="F10" t="n">
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
         <v>103.5550846014075</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto: Analysis complete | Temp: Ambient | Max Cycle: 98 | Anomalies: 0 | 2026-04-24 12:03
</commit_message>
<xml_diff>
--- a/reports/Master_Retention_Summary.xlsx
+++ b/reports/Master_Retention_Summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:F106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -513,10 +513,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>1.052322023911945</v>
+        <v>1.137456760812122</v>
       </c>
       <c r="C4" t="n">
-        <v>1.052322023911945</v>
+        <v>1.137456760812122</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>95.66563853744955</v>
+        <v>103.4051600738293</v>
       </c>
     </row>
     <row r="5">
@@ -537,10 +537,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>2.149665492833128</v>
+        <v>1.137011583397129</v>
       </c>
       <c r="C5" t="n">
-        <v>1.097343468921183</v>
+        <v>1.137011583397129</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>99.75849717465297</v>
+        <v>103.364689399739</v>
       </c>
     </row>
     <row r="6">
@@ -561,10 +561,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>3.245035743823332</v>
+        <v>2.273810507318694</v>
       </c>
       <c r="C6" t="n">
-        <v>1.095370250990204</v>
+        <v>1.136798923921565</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -577,7 +577,7 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>99.57911372638219</v>
+        <v>103.3453567201422</v>
       </c>
     </row>
     <row r="7">
@@ -585,10 +585,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>4.3427396829912</v>
+        <v>3.406011953491648</v>
       </c>
       <c r="C7" t="n">
-        <v>1.097703939167868</v>
+        <v>1.132201446172954</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -601,7 +601,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>99.79126719707895</v>
+        <v>102.9274041975413</v>
       </c>
     </row>
     <row r="8">
@@ -609,10 +609,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>5.438155466960088</v>
+        <v>4.535073167063902</v>
       </c>
       <c r="C8" t="n">
-        <v>1.095415783968887</v>
+        <v>1.129061213572254</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>99.58325308808065</v>
+        <v>102.6419285065685</v>
       </c>
     </row>
     <row r="9">
@@ -633,10 +633,10 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>6.408604373024617</v>
+        <v>5.65538205316819</v>
       </c>
       <c r="C9" t="n">
-        <v>0.9704489060645294</v>
+        <v>1.120308886104288</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -649,7 +649,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>88.22262782404812</v>
+        <v>101.8462623731171</v>
       </c>
     </row>
     <row r="10">
@@ -657,10 +657,10 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>7.495652225355175</v>
+        <v>6.765709906183314</v>
       </c>
       <c r="C10" t="n">
-        <v>1.087047852330558</v>
+        <v>1.110327853015124</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>98.82253203005074</v>
+        <v>100.9388957286477</v>
       </c>
     </row>
     <row r="11">
@@ -681,10 +681,10 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
-        <v>8.577396784697651</v>
+        <v>7.871236454520941</v>
       </c>
       <c r="C11" t="n">
-        <v>1.081744559342476</v>
+        <v>1.105526548337626</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -697,7 +697,7 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>98.34041448567962</v>
+        <v>100.5024134852387</v>
       </c>
     </row>
     <row r="12">
@@ -705,10 +705,10 @@
         <v>11</v>
       </c>
       <c r="B12" t="n">
-        <v>9.654946259914045</v>
+        <v>8.973180416597838</v>
       </c>
       <c r="C12" t="n">
-        <v>1.077549475216394</v>
+        <v>1.101943962076898</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -721,7 +721,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>97.95904320149033</v>
+        <v>100.1767238251725</v>
       </c>
     </row>
     <row r="13">
@@ -729,10 +729,10 @@
         <v>12</v>
       </c>
       <c r="B13" t="n">
-        <v>10.72613836450355</v>
+        <v>10.07175905337804</v>
       </c>
       <c r="C13" t="n">
-        <v>1.071192104589505</v>
+        <v>1.098578636780204</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -745,7 +745,7 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>97.38110041722771</v>
+        <v>99.87078516183668</v>
       </c>
     </row>
     <row r="14">
@@ -753,10 +753,10 @@
         <v>13</v>
       </c>
       <c r="B14" t="n">
-        <v>11.79860684954863</v>
+        <v>11.17652816931319</v>
       </c>
       <c r="C14" t="n">
-        <v>1.072468485045077</v>
+        <v>1.104769115935152</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -769,7 +769,7 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>97.49713500409788</v>
+        <v>100.4335559941048</v>
       </c>
     </row>
     <row r="15">
@@ -777,10 +777,10 @@
         <v>14</v>
       </c>
       <c r="B15" t="n">
-        <v>12.86786434001764</v>
+        <v>12.28214775502528</v>
       </c>
       <c r="C15" t="n">
-        <v>1.069257490469012</v>
+        <v>1.105619585712086</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -793,7 +793,7 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>97.20522640627377</v>
+        <v>100.5108714283714</v>
       </c>
     </row>
     <row r="16">
@@ -801,10 +801,10 @@
         <v>15</v>
       </c>
       <c r="B16" t="n">
-        <v>13.9297296638013</v>
+        <v>13.38758978184518</v>
       </c>
       <c r="C16" t="n">
-        <v>1.061865323783662</v>
+        <v>1.105442026819896</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -817,7 +817,7 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>96.53321125306019</v>
+        <v>100.4947297108996</v>
       </c>
     </row>
     <row r="17">
@@ -825,10 +825,10 @@
         <v>16</v>
       </c>
       <c r="B17" t="n">
-        <v>14.98952004353151</v>
+        <v>14.49259840940244</v>
       </c>
       <c r="C17" t="n">
-        <v>1.05979037973021</v>
+        <v>1.105008627557268</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -841,7 +841,7 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>96.34457997547359</v>
+        <v>100.4553297779335</v>
       </c>
     </row>
     <row r="18">
@@ -849,10 +849,10 @@
         <v>17</v>
       </c>
       <c r="B18" t="n">
-        <v>16.04749855873573</v>
+        <v>15.59690381478543</v>
       </c>
       <c r="C18" t="n">
-        <v>1.057978515204223</v>
+        <v>1.104305405382988</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -865,7 +865,7 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>96.17986501856569</v>
+        <v>100.3914004893625</v>
       </c>
     </row>
     <row r="19">
@@ -873,10 +873,10 @@
         <v>18</v>
       </c>
       <c r="B19" t="n">
-        <v>17.10340536937683</v>
+        <v>16.70080671099171</v>
       </c>
       <c r="C19" t="n">
-        <v>1.055906810641098</v>
+        <v>1.103902896206275</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -889,7 +889,7 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>95.99152824009978</v>
+        <v>100.354808746025</v>
       </c>
     </row>
     <row r="20">
@@ -897,10 +897,10 @@
         <v>19</v>
       </c>
       <c r="B20" t="n">
-        <v>18.1556290521891</v>
+        <v>17.80416451293284</v>
       </c>
       <c r="C20" t="n">
-        <v>1.052223682812269</v>
+        <v>1.103357801941137</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -913,7 +913,7 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>95.65669843747897</v>
+        <v>100.3052547219215</v>
       </c>
     </row>
     <row r="21">
@@ -921,10 +921,10 @@
         <v>20</v>
       </c>
       <c r="B21" t="n">
-        <v>19.20997154058639</v>
+        <v>18.9066816254796</v>
       </c>
       <c r="C21" t="n">
-        <v>1.054342488397296</v>
+        <v>1.102517112546753</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -937,7 +937,7 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>95.84931712702691</v>
+        <v>100.2288284133412</v>
       </c>
     </row>
     <row r="22">
@@ -945,10 +945,10 @@
         <v>21</v>
       </c>
       <c r="B22" t="n">
-        <v>20.26299732771692</v>
+        <v>20.00835414851035</v>
       </c>
       <c r="C22" t="n">
-        <v>1.053025787130522</v>
+        <v>1.101672523030757</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -961,7 +961,7 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>95.72961701186567</v>
+        <v>100.1520475482506</v>
       </c>
     </row>
     <row r="23">
@@ -969,10 +969,10 @@
         <v>22</v>
       </c>
       <c r="B23" t="n">
-        <v>21.31033341195971</v>
+        <v>21.10929865392855</v>
       </c>
       <c r="C23" t="n">
-        <v>1.047336084242794</v>
+        <v>1.100944505418198</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -985,7 +985,7 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>95.21237129479941</v>
+        <v>100.0858641289271</v>
       </c>
     </row>
     <row r="24">
@@ -993,10 +993,10 @@
         <v>23</v>
       </c>
       <c r="B24" t="n">
-        <v>22.35610598333428</v>
+        <v>22.20935616007882</v>
       </c>
       <c r="C24" t="n">
-        <v>1.045772571374567</v>
+        <v>1.100057506150264</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1009,7 +1009,7 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>95.07023376132425</v>
+        <v>100.0052278318422</v>
       </c>
     </row>
     <row r="25">
@@ -1017,10 +1017,10 @@
         <v>24</v>
       </c>
       <c r="B25" t="n">
-        <v>23.40056677922347</v>
+        <v>23.30885072692595</v>
       </c>
       <c r="C25" t="n">
-        <v>1.044460795889197</v>
+        <v>1.099494566847138</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1033,7 +1033,7 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>94.95098144447246</v>
+        <v>99.95405153155799</v>
       </c>
     </row>
     <row r="26">
@@ -1041,10 +1041,10 @@
         <v>25</v>
       </c>
       <c r="B26" t="n">
-        <v>24.44359582009594</v>
+        <v>24.40767121329099</v>
       </c>
       <c r="C26" t="n">
-        <v>1.043029040872465</v>
+        <v>1.098820486365039</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1057,7 +1057,7 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>94.82082189749683</v>
+        <v>99.8927714877308</v>
       </c>
     </row>
     <row r="27">
@@ -1065,10 +1065,10 @@
         <v>26</v>
       </c>
       <c r="B27" t="n">
-        <v>25.4831948218273</v>
+        <v>25.50586794777845</v>
       </c>
       <c r="C27" t="n">
-        <v>1.039599001731357</v>
+        <v>1.098196734487459</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -1081,7 +1081,7 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>94.5090001573961</v>
+        <v>99.83606677158717</v>
       </c>
     </row>
     <row r="28">
@@ -1089,10 +1089,10 @@
         <v>27</v>
       </c>
       <c r="B28" t="n">
-        <v>26.52631445530069</v>
+        <v>26.60321975865625</v>
       </c>
       <c r="C28" t="n">
-        <v>1.043119633473388</v>
+        <v>1.097351810877797</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -1105,7 +1105,7 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>94.82905758848985</v>
+        <v>99.75925553434514</v>
       </c>
     </row>
     <row r="29">
@@ -1113,10 +1113,10 @@
         <v>28</v>
       </c>
       <c r="B29" t="n">
-        <v>27.5686670992941</v>
+        <v>27.69924910305312</v>
       </c>
       <c r="C29" t="n">
-        <v>1.042352643993418</v>
+        <v>1.096029344396872</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -1129,7 +1129,7 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>94.75933127212889</v>
+        <v>99.63903130880651</v>
       </c>
     </row>
     <row r="30">
@@ -1137,10 +1137,10 @@
         <v>29</v>
       </c>
       <c r="B30" t="n">
-        <v>28.60979222529076</v>
+        <v>28.78304771385524</v>
       </c>
       <c r="C30" t="n">
-        <v>1.041125125996658</v>
+        <v>1.08379861080212</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -1153,7 +1153,7 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>94.64773872696887</v>
+        <v>98.52714643655634</v>
       </c>
     </row>
     <row r="31">
@@ -1161,10 +1161,10 @@
         <v>30</v>
       </c>
       <c r="B31" t="n">
-        <v>29.64938541586051</v>
+        <v>29.86089125304247</v>
       </c>
       <c r="C31" t="n">
-        <v>1.03959319056975</v>
+        <v>1.077843539187231</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -1177,7 +1177,7 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>94.50847186997728</v>
+        <v>97.9857762897483</v>
       </c>
     </row>
     <row r="32">
@@ -1185,10 +1185,10 @@
         <v>31</v>
       </c>
       <c r="B32" t="n">
-        <v>30.68792447367722</v>
+        <v>30.93516370280259</v>
       </c>
       <c r="C32" t="n">
-        <v>1.038539057816706</v>
+        <v>1.074272449760119</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -1201,7 +1201,7 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>94.41264161970055</v>
+        <v>97.66113179637449</v>
       </c>
     </row>
     <row r="33">
@@ -1209,10 +1209,10 @@
         <v>32</v>
       </c>
       <c r="B33" t="n">
-        <v>31.7263162152612</v>
+        <v>32.00667863670272</v>
       </c>
       <c r="C33" t="n">
-        <v>1.038391741583983</v>
+        <v>1.071514933900133</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -1225,7 +1225,7 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>94.39924923490749</v>
+        <v>97.41044853637571</v>
       </c>
     </row>
     <row r="34">
@@ -1233,10 +1233,10 @@
         <v>33</v>
       </c>
       <c r="B34" t="n">
-        <v>32.76338812831584</v>
+        <v>33.0767579630373</v>
       </c>
       <c r="C34" t="n">
-        <v>1.037071913054639</v>
+        <v>1.070079326334579</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -1249,7 +1249,7 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>94.27926482314901</v>
+        <v>97.27993875768897</v>
       </c>
     </row>
     <row r="35">
@@ -1257,10 +1257,10 @@
         <v>34</v>
       </c>
       <c r="B35" t="n">
-        <v>33.7987298481729</v>
+        <v>34.15648554158277</v>
       </c>
       <c r="C35" t="n">
-        <v>1.035341719857065</v>
+        <v>1.079727578545466</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -1273,7 +1273,7 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>94.12197453246048</v>
+        <v>98.15705259504234</v>
       </c>
     </row>
     <row r="36">
@@ -1281,10 +1281,10 @@
         <v>35</v>
       </c>
       <c r="B36" t="n">
-        <v>34.83270037940027</v>
+        <v>35.23833022797701</v>
       </c>
       <c r="C36" t="n">
-        <v>1.033970531227368</v>
+        <v>1.081844686394241</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -1297,7 +1297,7 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>93.9973210206698</v>
+        <v>98.34951694493101</v>
       </c>
     </row>
     <row r="37">
@@ -1305,10 +1305,10 @@
         <v>36</v>
       </c>
       <c r="B37" t="n">
-        <v>35.86574666724295</v>
+        <v>36.30958559777886</v>
       </c>
       <c r="C37" t="n">
-        <v>1.033046287842673</v>
+        <v>1.071255369801854</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -1321,7 +1321,7 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>93.91329889478844</v>
+        <v>97.38685180016853</v>
       </c>
     </row>
     <row r="38">
@@ -1329,10 +1329,10 @@
         <v>37</v>
       </c>
       <c r="B38" t="n">
-        <v>36.89740618197521</v>
+        <v>37.37492471677352</v>
       </c>
       <c r="C38" t="n">
-        <v>1.031659514732269</v>
+        <v>1.065339118994657</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -1345,7 +1345,7 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>93.78722861202442</v>
+        <v>96.84901081769613</v>
       </c>
     </row>
     <row r="39">
@@ -1353,10 +1353,10 @@
         <v>38</v>
       </c>
       <c r="B39" t="n">
-        <v>37.92829661484846</v>
+        <v>38.43806126470225</v>
       </c>
       <c r="C39" t="n">
-        <v>1.030890432873242</v>
+        <v>1.063136547928728</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -1369,7 +1369,7 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>93.71731207938568</v>
+        <v>96.64877708442984</v>
       </c>
     </row>
     <row r="40">
@@ -1377,10 +1377,10 @@
         <v>39</v>
       </c>
       <c r="B40" t="n">
-        <v>38.95850830029624</v>
+        <v>39.49974416627123</v>
       </c>
       <c r="C40" t="n">
-        <v>1.030211685447789</v>
+        <v>1.061682901568986</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -1393,7 +1393,7 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>93.65560776798078</v>
+        <v>96.51662741536235</v>
       </c>
     </row>
     <row r="41">
@@ -1401,10 +1401,10 @@
         <v>40</v>
       </c>
       <c r="B41" t="n">
-        <v>39.98860228884588</v>
+        <v>40.56061757267415</v>
       </c>
       <c r="C41" t="n">
-        <v>1.030093988549631</v>
+        <v>1.060873406402912</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
@@ -1417,7 +1417,7 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>93.6449080499664</v>
+        <v>96.44303694571929</v>
       </c>
     </row>
     <row r="42">
@@ -1425,10 +1425,10 @@
         <v>41</v>
       </c>
       <c r="B42" t="n">
-        <v>41.01705848167371</v>
+        <v>41.63114874496969</v>
       </c>
       <c r="C42" t="n">
-        <v>1.028456192827839</v>
+        <v>1.070531172295539</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -1441,7 +1441,7 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>93.49601752980357</v>
+        <v>97.32101566323078</v>
       </c>
     </row>
     <row r="43">
@@ -1449,10 +1449,10 @@
         <v>42</v>
       </c>
       <c r="B43" t="n">
-        <v>42.04438475344786</v>
+        <v>42.70383388345945</v>
       </c>
       <c r="C43" t="n">
-        <v>1.027326271774143</v>
+        <v>1.07268513848976</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -1465,7 +1465,7 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>93.39329743401301</v>
+        <v>97.51683077179636</v>
       </c>
     </row>
     <row r="44">
@@ -1473,10 +1473,10 @@
         <v>43</v>
       </c>
       <c r="B44" t="n">
-        <v>43.07010828743945</v>
+        <v>43.76889004370484</v>
       </c>
       <c r="C44" t="n">
-        <v>1.025723533991588</v>
+        <v>1.065056160245398</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -1489,7 +1489,7 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>93.24759399923526</v>
+        <v>96.82328729503614</v>
       </c>
     </row>
     <row r="45">
@@ -1497,10 +1497,10 @@
         <v>44</v>
       </c>
       <c r="B45" t="n">
-        <v>44.08658300417674</v>
+        <v>44.82625898474644</v>
       </c>
       <c r="C45" t="n">
-        <v>1.016474716737292</v>
+        <v>1.057368941041595</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -1513,7 +1513,7 @@
         </is>
       </c>
       <c r="F45" t="n">
-        <v>92.40679243066293</v>
+        <v>96.12444918559956</v>
       </c>
     </row>
     <row r="46">
@@ -1521,10 +1521,10 @@
         <v>45</v>
       </c>
       <c r="B46" t="n">
-        <v>45.10024541836556</v>
+        <v>45.88284822358288</v>
       </c>
       <c r="C46" t="n">
-        <v>1.013662414188822</v>
+        <v>1.056589238836445</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -1537,7 +1537,7 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>92.15112856262017</v>
+        <v>96.05356716694951</v>
       </c>
     </row>
     <row r="47">
@@ -1545,10 +1545,10 @@
         <v>46</v>
       </c>
       <c r="B47" t="n">
-        <v>46.1126554106551</v>
+        <v>46.93851289681216</v>
       </c>
       <c r="C47" t="n">
-        <v>1.012409992289541</v>
+        <v>1.05566467322928</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
@@ -1561,7 +1561,7 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>92.03727202632192</v>
+        <v>95.96951574811639</v>
       </c>
     </row>
     <row r="48">
@@ -1569,10 +1569,10 @@
         <v>47</v>
       </c>
       <c r="B48" t="n">
-        <v>46.39238602108801</v>
+        <v>47.9926422861599</v>
       </c>
       <c r="C48" t="n">
-        <v>0.2797306104329067</v>
+        <v>1.054129389347736</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
@@ -1585,22 +1585,22 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>25.4300554939006</v>
+        <v>95.8299444861578</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>1</v>
+        <v>48</v>
       </c>
       <c r="B49" t="n">
-        <v>1.160620725192767</v>
+        <v>49.05435303477396</v>
       </c>
       <c r="C49" t="n">
-        <v>1.160620725192767</v>
+        <v>1.061710748614061</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>CS2_36</t>
+          <t>CS2_35</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -1609,22 +1609,22 @@
         </is>
       </c>
       <c r="F49" t="n">
-        <v>105.5109750175243</v>
+        <v>96.51915896491464</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>2</v>
+        <v>49</v>
       </c>
       <c r="B50" t="n">
-        <v>1.145706012058183</v>
+        <v>50.11919434062645</v>
       </c>
       <c r="C50" t="n">
-        <v>1.145706012058183</v>
+        <v>1.064841305852489</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>CS2_36</t>
+          <t>CS2_35</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -1633,22 +1633,22 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>104.1550920052894</v>
+        <v>96.80375507749903</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="B51" t="n">
-        <v>1.153332504667897</v>
+        <v>51.18325301816826</v>
       </c>
       <c r="C51" t="n">
-        <v>1.153332504667897</v>
+        <v>1.064058677541809</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>CS2_37</t>
+          <t>CS2_35</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -1657,22 +1657,22 @@
         </is>
       </c>
       <c r="F51" t="n">
-        <v>104.8484095152634</v>
+        <v>96.73260704925532</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>2</v>
+        <v>51</v>
       </c>
       <c r="B52" t="n">
-        <v>1.134444845802931</v>
+        <v>52.23606753857995</v>
       </c>
       <c r="C52" t="n">
-        <v>1.134444845802931</v>
+        <v>1.052814520411694</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>CS2_37</t>
+          <t>CS2_35</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -1681,22 +1681,22 @@
         </is>
       </c>
       <c r="F52" t="n">
-        <v>103.1313496184483</v>
+        <v>95.71041094651763</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>1</v>
+        <v>52</v>
       </c>
       <c r="B53" t="n">
-        <v>1.16241194625815</v>
+        <v>53.28768827080705</v>
       </c>
       <c r="C53" t="n">
-        <v>1.16241194625815</v>
+        <v>1.0516207322271</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>CS2_38</t>
+          <t>CS2_35</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -1705,22 +1705,22 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>105.6738132961954</v>
+        <v>95.60188474791818</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>2</v>
+        <v>53</v>
       </c>
       <c r="B54" t="n">
-        <v>1.140773820517232</v>
+        <v>54.33830268728399</v>
       </c>
       <c r="C54" t="n">
-        <v>1.140773820517232</v>
+        <v>1.05061441647694</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>CS2_38</t>
+          <t>CS2_35</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -1729,30 +1729,1254 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>103.706710956112</v>
+        <v>95.51040149790359</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" t="n">
+        <v>1.052322023911945</v>
+      </c>
+      <c r="C55" t="n">
+        <v>1.052322023911945</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>95.66563853744955</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" t="n">
+        <v>2.149665492833128</v>
+      </c>
+      <c r="C56" t="n">
+        <v>1.097343468921183</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F56" t="n">
+        <v>99.75849717465297</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" t="n">
+        <v>3.245035743823332</v>
+      </c>
+      <c r="C57" t="n">
+        <v>1.095370250990204</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F57" t="n">
+        <v>99.57911372638219</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" t="n">
+        <v>4.3427396829912</v>
+      </c>
+      <c r="C58" t="n">
+        <v>1.097703939167868</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F58" t="n">
+        <v>99.79126719707895</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" t="n">
+        <v>5.438155466960088</v>
+      </c>
+      <c r="C59" t="n">
+        <v>1.095415783968887</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F59" t="n">
+        <v>99.58325308808065</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" t="n">
+        <v>6.408604373024617</v>
+      </c>
+      <c r="C60" t="n">
+        <v>0.9704489060645294</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F60" t="n">
+        <v>88.22262782404812</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" t="n">
+        <v>7.495652225355175</v>
+      </c>
+      <c r="C61" t="n">
+        <v>1.087047852330558</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F61" t="n">
+        <v>98.82253203005074</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" t="n">
+        <v>8.577396784697651</v>
+      </c>
+      <c r="C62" t="n">
+        <v>1.081744559342476</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F62" t="n">
+        <v>98.34041448567962</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" t="n">
+        <v>9.654946259914045</v>
+      </c>
+      <c r="C63" t="n">
+        <v>1.077549475216394</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F63" t="n">
+        <v>97.95904320149033</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" t="n">
+        <v>10.72613836450355</v>
+      </c>
+      <c r="C64" t="n">
+        <v>1.071192104589505</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F64" t="n">
+        <v>97.38110041722771</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" t="n">
+        <v>11.79860684954863</v>
+      </c>
+      <c r="C65" t="n">
+        <v>1.072468485045077</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F65" t="n">
+        <v>97.49713500409788</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" t="n">
+        <v>12.86786434001764</v>
+      </c>
+      <c r="C66" t="n">
+        <v>1.069257490469012</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F66" t="n">
+        <v>97.20522640627377</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" t="n">
+        <v>13.9297296638013</v>
+      </c>
+      <c r="C67" t="n">
+        <v>1.061865323783662</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F67" t="n">
+        <v>96.53321125306019</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" t="n">
+        <v>14.98952004353151</v>
+      </c>
+      <c r="C68" t="n">
+        <v>1.05979037973021</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F68" t="n">
+        <v>96.34457997547359</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" t="n">
+        <v>16.04749855873573</v>
+      </c>
+      <c r="C69" t="n">
+        <v>1.057978515204223</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F69" t="n">
+        <v>96.17986501856569</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" t="n">
+        <v>17.10340536937683</v>
+      </c>
+      <c r="C70" t="n">
+        <v>1.055906810641098</v>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F70" t="n">
+        <v>95.99152824009978</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" t="n">
+        <v>18.1556290521891</v>
+      </c>
+      <c r="C71" t="n">
+        <v>1.052223682812269</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F71" t="n">
+        <v>95.65669843747897</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" t="n">
+        <v>19.20997154058639</v>
+      </c>
+      <c r="C72" t="n">
+        <v>1.054342488397296</v>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F72" t="n">
+        <v>95.84931712702691</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" t="n">
+        <v>20.26299732771692</v>
+      </c>
+      <c r="C73" t="n">
+        <v>1.053025787130522</v>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F73" t="n">
+        <v>95.72961701186567</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" t="n">
+        <v>21.31033341195971</v>
+      </c>
+      <c r="C74" t="n">
+        <v>1.047336084242794</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F74" t="n">
+        <v>95.21237129479941</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" t="n">
+        <v>22.35610598333428</v>
+      </c>
+      <c r="C75" t="n">
+        <v>1.045772571374567</v>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F75" t="n">
+        <v>95.07023376132425</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" t="n">
+        <v>23.40056677922347</v>
+      </c>
+      <c r="C76" t="n">
+        <v>1.044460795889197</v>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F76" t="n">
+        <v>94.95098144447246</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" t="n">
+        <v>24.44359582009594</v>
+      </c>
+      <c r="C77" t="n">
+        <v>1.043029040872465</v>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F77" t="n">
+        <v>94.82082189749683</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" t="n">
+        <v>25.4831948218273</v>
+      </c>
+      <c r="C78" t="n">
+        <v>1.039599001731357</v>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F78" t="n">
+        <v>94.5090001573961</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" t="n">
+        <v>26.52631445530069</v>
+      </c>
+      <c r="C79" t="n">
+        <v>1.043119633473388</v>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F79" t="n">
+        <v>94.82905758848985</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" t="n">
+        <v>27.5686670992941</v>
+      </c>
+      <c r="C80" t="n">
+        <v>1.042352643993418</v>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F80" t="n">
+        <v>94.75933127212889</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" t="n">
+        <v>28.60979222529076</v>
+      </c>
+      <c r="C81" t="n">
+        <v>1.041125125996658</v>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F81" t="n">
+        <v>94.64773872696887</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" t="n">
+        <v>29.64938541586051</v>
+      </c>
+      <c r="C82" t="n">
+        <v>1.03959319056975</v>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F82" t="n">
+        <v>94.50847186997728</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" t="n">
+        <v>30.68792447367722</v>
+      </c>
+      <c r="C83" t="n">
+        <v>1.038539057816706</v>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F83" t="n">
+        <v>94.41264161970055</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" t="n">
+        <v>31.7263162152612</v>
+      </c>
+      <c r="C84" t="n">
+        <v>1.038391741583983</v>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F84" t="n">
+        <v>94.39924923490749</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" t="n">
+        <v>32.76338812831584</v>
+      </c>
+      <c r="C85" t="n">
+        <v>1.037071913054639</v>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F85" t="n">
+        <v>94.27926482314901</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" t="n">
+        <v>33.7987298481729</v>
+      </c>
+      <c r="C86" t="n">
+        <v>1.035341719857065</v>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F86" t="n">
+        <v>94.12197453246048</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" t="n">
+        <v>34.83270037940027</v>
+      </c>
+      <c r="C87" t="n">
+        <v>1.033970531227368</v>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F87" t="n">
+        <v>93.9973210206698</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" t="n">
+        <v>35.86574666724295</v>
+      </c>
+      <c r="C88" t="n">
+        <v>1.033046287842673</v>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F88" t="n">
+        <v>93.91329889478844</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" t="n">
+        <v>36.89740618197521</v>
+      </c>
+      <c r="C89" t="n">
+        <v>1.031659514732269</v>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F89" t="n">
+        <v>93.78722861202442</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" t="n">
+        <v>37.92829661484846</v>
+      </c>
+      <c r="C90" t="n">
+        <v>1.030890432873242</v>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F90" t="n">
+        <v>93.71731207938568</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" t="n">
+        <v>38.95850830029624</v>
+      </c>
+      <c r="C91" t="n">
+        <v>1.030211685447789</v>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F91" t="n">
+        <v>93.65560776798078</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" t="n">
+        <v>39.98860228884588</v>
+      </c>
+      <c r="C92" t="n">
+        <v>1.030093988549631</v>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F92" t="n">
+        <v>93.6449080499664</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" t="n">
+        <v>41.01705848167371</v>
+      </c>
+      <c r="C93" t="n">
+        <v>1.028456192827839</v>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F93" t="n">
+        <v>93.49601752980357</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" t="n">
+        <v>42.04438475344786</v>
+      </c>
+      <c r="C94" t="n">
+        <v>1.027326271774143</v>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F94" t="n">
+        <v>93.39329743401301</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" t="n">
+        <v>43.07010828743945</v>
+      </c>
+      <c r="C95" t="n">
+        <v>1.025723533991588</v>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F95" t="n">
+        <v>93.24759399923526</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" t="n">
+        <v>44.08658300417674</v>
+      </c>
+      <c r="C96" t="n">
+        <v>1.016474716737292</v>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F96" t="n">
+        <v>92.40679243066293</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" t="n">
+        <v>45.10024541836556</v>
+      </c>
+      <c r="C97" t="n">
+        <v>1.013662414188822</v>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F97" t="n">
+        <v>92.15112856262017</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>97</v>
+      </c>
+      <c r="B98" t="n">
+        <v>46.1126554106551</v>
+      </c>
+      <c r="C98" t="n">
+        <v>1.012409992289541</v>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F98" t="n">
+        <v>92.03727202632192</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>98</v>
+      </c>
+      <c r="B99" t="n">
+        <v>46.39238602108801</v>
+      </c>
+      <c r="C99" t="n">
+        <v>0.2797306104329067</v>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>CS2_35</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F99" t="n">
+        <v>25.4300554939006</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>1</v>
+      </c>
+      <c r="B100" t="n">
+        <v>1.160620725192767</v>
+      </c>
+      <c r="C100" t="n">
+        <v>1.160620725192767</v>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>CS2_36</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F100" t="n">
+        <v>105.5109750175243</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>2</v>
+      </c>
+      <c r="B101" t="n">
+        <v>1.145706012058183</v>
+      </c>
+      <c r="C101" t="n">
+        <v>1.145706012058183</v>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>CS2_36</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F101" t="n">
+        <v>104.1550920052894</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>1</v>
+      </c>
+      <c r="B102" t="n">
+        <v>1.153332504667897</v>
+      </c>
+      <c r="C102" t="n">
+        <v>1.153332504667897</v>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>CS2_37</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F102" t="n">
+        <v>104.8484095152634</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>2</v>
+      </c>
+      <c r="B103" t="n">
+        <v>1.134444845802931</v>
+      </c>
+      <c r="C103" t="n">
+        <v>1.134444845802931</v>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>CS2_37</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F103" t="n">
+        <v>103.1313496184483</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>1</v>
+      </c>
+      <c r="B104" t="n">
+        <v>1.16241194625815</v>
+      </c>
+      <c r="C104" t="n">
+        <v>1.16241194625815</v>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F104" t="n">
+        <v>105.6738132961954</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>2</v>
+      </c>
+      <c r="B105" t="n">
+        <v>1.140773820517232</v>
+      </c>
+      <c r="C105" t="n">
+        <v>1.140773820517232</v>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>CS2_38</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F105" t="n">
+        <v>103.706710956112</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
         <v>3</v>
       </c>
-      <c r="B55" t="n">
+      <c r="B106" t="n">
         <v>1.139105930615482</v>
       </c>
-      <c r="C55" t="n">
+      <c r="C106" t="n">
         <v>1.139105930615482</v>
       </c>
-      <c r="D55" t="inlineStr">
+      <c r="D106" t="inlineStr">
         <is>
           <t>CS2_38</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>Ambient</t>
-        </is>
-      </c>
-      <c r="F55" t="n">
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Ambient</t>
+        </is>
+      </c>
+      <c r="F106" t="n">
         <v>103.5550846014075</v>
       </c>
     </row>

</xml_diff>